<commit_message>
docs: Document Excel native Undo limitations and custom patch behavior
</commit_message>
<xml_diff>
--- a/reference/Form/Stores.xlsx
+++ b/reference/Form/Stores.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f85608126126f9cf/桌面/AlchemyPlanning/Form/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Project\ExcelEnumSelectionTool\reference\Form\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="682" documentId="13_ncr:1_{B6440DA5-C8D0-4687-9755-5BAE39931679}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CC653871-D1CA-4C1C-86DC-7165D2CA0F2D}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE058C5A-E1CC-4055-A398-ABF435946C5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E5E47801-C43D-4B4D-802B-23CF1146FAE0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E5E47801-C43D-4B4D-802B-23CF1146FAE0}"/>
   </bookViews>
   <sheets>
     <sheet name="#Info" sheetId="1" r:id="rId1"/>
@@ -753,7 +753,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -866,7 +866,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="一般" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -886,7 +886,6 @@
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <xxl21:alternateUrls>
       <xxl21:absoluteUrl r:id="rId2"/>
-      <xxl21:relativeUrl r:id="rId3"/>
     </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="範例"/>
@@ -982,14 +981,17 @@
       <sheetName val="#Info"/>
       <sheetName val="Element"/>
       <sheetName val="YinYang"/>
+      <sheetName val="MaterialState"/>
       <sheetName val="Material"/>
       <sheetName val="#備份"/>
+      <sheetName val="PestleMortar"/>
     </sheetNames>
     <sheetDataSet>
       <sheetData sheetId="0"/>
       <sheetData sheetId="1"/>
       <sheetData sheetId="2"/>
-      <sheetData sheetId="3">
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4">
         <row r="1">
           <cell r="B1" t="str">
             <v>#名稱</v>
@@ -998,7 +1000,7 @@
             <v>材料ID</v>
           </cell>
           <cell r="E1" t="str">
-            <v>#解鎖等級</v>
+            <v>材料顏色</v>
           </cell>
         </row>
         <row r="2">
@@ -1009,11 +1011,15 @@
             <v>MaterialID</v>
           </cell>
           <cell r="E2" t="str">
-            <v>LevelReq</v>
+            <v>ColorHex</v>
           </cell>
         </row>
         <row r="3">
+          <cell r="B3"/>
           <cell r="C3" t="str">
+            <v>string</v>
+          </cell>
+          <cell r="E3" t="str">
             <v>string</v>
           </cell>
         </row>
@@ -1022,10 +1028,10 @@
             <v>黑鉛</v>
           </cell>
           <cell r="C4" t="str">
-            <v>230101</v>
+            <v>101001</v>
           </cell>
           <cell r="E4" t="str">
-            <v>01</v>
+            <v>2F353B</v>
           </cell>
         </row>
         <row r="5">
@@ -1033,10 +1039,10 @@
             <v>水銀</v>
           </cell>
           <cell r="C5" t="str">
-            <v>230102</v>
+            <v>101002</v>
           </cell>
           <cell r="E5" t="str">
-            <v>01</v>
+            <v>E5E4E2</v>
           </cell>
         </row>
         <row r="6">
@@ -1044,10 +1050,10 @@
             <v>丹砂</v>
           </cell>
           <cell r="C6" t="str">
-            <v>230103</v>
+            <v>101003</v>
           </cell>
           <cell r="E6" t="str">
-            <v>01</v>
+            <v>E34234</v>
           </cell>
         </row>
         <row r="7">
@@ -1055,10 +1061,10 @@
             <v>曾青</v>
           </cell>
           <cell r="C7" t="str">
-            <v>230104</v>
+            <v>101004</v>
           </cell>
           <cell r="E7" t="str">
-            <v>01</v>
+            <v>40E0D0</v>
           </cell>
         </row>
         <row r="8">
@@ -1066,10 +1072,10 @@
             <v>石膏</v>
           </cell>
           <cell r="C8" t="str">
-            <v>230105</v>
+            <v>101005</v>
           </cell>
           <cell r="E8" t="str">
-            <v>01</v>
+            <v>FFFFFF</v>
           </cell>
         </row>
         <row r="9">
@@ -1077,10 +1083,10 @@
             <v>雄黃</v>
           </cell>
           <cell r="C9" t="str">
-            <v>230106</v>
+            <v>101006</v>
           </cell>
           <cell r="E9" t="str">
-            <v>01</v>
+            <v>FFA500</v>
           </cell>
         </row>
         <row r="10">
@@ -1088,10 +1094,10 @@
             <v>硝石</v>
           </cell>
           <cell r="C10" t="str">
-            <v>230201</v>
+            <v>102001</v>
           </cell>
           <cell r="E10" t="str">
-            <v>02</v>
+            <v>EDEFF2</v>
           </cell>
         </row>
         <row r="11">
@@ -1099,10 +1105,10 @@
             <v>石硫黃</v>
           </cell>
           <cell r="C11" t="str">
-            <v>230202</v>
+            <v>102002</v>
           </cell>
           <cell r="E11" t="str">
-            <v>02</v>
+            <v>FDFD96</v>
           </cell>
         </row>
         <row r="12">
@@ -1110,10 +1116,10 @@
             <v>鐘乳石</v>
           </cell>
           <cell r="C12" t="str">
-            <v>230203</v>
+            <v>102003</v>
           </cell>
           <cell r="E12" t="str">
-            <v>02</v>
+            <v>FBFBE8</v>
           </cell>
         </row>
         <row r="13">
@@ -1121,10 +1127,10 @@
             <v>銅</v>
           </cell>
           <cell r="C13" t="str">
-            <v>230301</v>
+            <v>103001</v>
           </cell>
           <cell r="E13" t="str">
-            <v>03</v>
+            <v>B87333</v>
           </cell>
         </row>
         <row r="14">
@@ -1132,10 +1138,10 @@
             <v>黃金</v>
           </cell>
           <cell r="C14" t="str">
-            <v>230302</v>
+            <v>103002</v>
           </cell>
           <cell r="E14" t="str">
-            <v>03</v>
+            <v>FFD700</v>
           </cell>
         </row>
         <row r="15">
@@ -1143,10 +1149,10 @@
             <v>白玉</v>
           </cell>
           <cell r="C15" t="str">
-            <v>230401</v>
+            <v>104001</v>
           </cell>
           <cell r="E15" t="str">
-            <v>04</v>
+            <v>F5F5F0</v>
           </cell>
         </row>
         <row r="16">
@@ -1154,10 +1160,10 @@
             <v>雲母</v>
           </cell>
           <cell r="C16" t="str">
-            <v>230402</v>
+            <v>104002</v>
           </cell>
           <cell r="E16" t="str">
-            <v>04</v>
+            <v>E6E8EC</v>
           </cell>
         </row>
         <row r="17">
@@ -1165,10 +1171,10 @@
             <v>白石英</v>
           </cell>
           <cell r="C17" t="str">
-            <v>230403</v>
+            <v>104003</v>
           </cell>
           <cell r="E17" t="str">
-            <v>04</v>
+            <v>F0F8FF</v>
           </cell>
         </row>
         <row r="18">
@@ -1176,10 +1182,10 @@
             <v>磁石</v>
           </cell>
           <cell r="C18" t="str">
-            <v>230501</v>
+            <v>105001</v>
           </cell>
           <cell r="E18" t="str">
-            <v>05</v>
+            <v>4A4A4A</v>
           </cell>
         </row>
         <row r="19">
@@ -1187,10 +1193,10 @@
             <v>殞鐵</v>
           </cell>
           <cell r="C19" t="str">
-            <v>230502</v>
+            <v>105002</v>
           </cell>
           <cell r="E19" t="str">
-            <v>05</v>
+            <v>1C1C1C</v>
           </cell>
         </row>
         <row r="20">
@@ -1198,10 +1204,10 @@
             <v>松煙</v>
           </cell>
           <cell r="C20" t="str">
-            <v>230503</v>
+            <v>105003</v>
           </cell>
           <cell r="E20" t="str">
-            <v>05</v>
+            <v>2B2B2B</v>
           </cell>
         </row>
         <row r="21">
@@ -1209,10 +1215,10 @@
             <v>空青</v>
           </cell>
           <cell r="C21" t="str">
-            <v>230504</v>
+            <v>105004</v>
           </cell>
           <cell r="E21" t="str">
-            <v>05</v>
+            <v>2FA4A9</v>
           </cell>
         </row>
         <row r="22">
@@ -1220,10 +1226,10 @@
             <v>紫石英</v>
           </cell>
           <cell r="C22" t="str">
-            <v>230601</v>
-          </cell>
-          <cell r="E22" t="str">
-            <v>06</v>
+            <v>106001</v>
+          </cell>
+          <cell r="E22">
+            <v>800080</v>
           </cell>
         </row>
         <row r="23">
@@ -1231,25 +1237,22 @@
             <v>赤石脂</v>
           </cell>
           <cell r="C23" t="str">
-            <v>230602</v>
+            <v>106002</v>
           </cell>
           <cell r="E23" t="str">
-            <v>06</v>
+            <v>9C3A2B</v>
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 佈景主題">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1566,77 +1569,77 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D881636-3FCB-4293-936C-4A4F328197BA}">
   <dimension ref="A1:A24"/>
-  <sheetFormatPr defaultRowHeight="12.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="16384" width="8.88671875" style="1"/>
+    <col min="1" max="16384" width="8.875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1">
       <c r="A2" s="1" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1">
       <c r="A4" s="1" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1">
       <c r="A5" s="1" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:1">
       <c r="A9" s="1" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:1">
       <c r="A10" s="1" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:1">
       <c r="A11" s="1" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:1">
       <c r="A13" s="1" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:1">
       <c r="A15" s="1" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:1">
       <c r="A17" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:1">
       <c r="A20" s="1" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:1">
       <c r="A22" s="1" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:1">
       <c r="A24" s="1" t="s">
         <v>150</v>
       </c>
@@ -1650,24 +1653,24 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7324E2FE-99BE-4C1F-9D48-4400248D69B0}">
   <dimension ref="A1:M33"/>
-  <sheetFormatPr defaultRowHeight="12.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="7.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="3.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="18.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.33203125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="15.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="21.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="8.88671875" style="1"/>
+    <col min="1" max="1" width="7.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="3.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="18.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="15.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.25" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="21.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="16384" width="8.875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13">
       <c r="A1" s="3" t="s">
         <v>2</v>
       </c>
@@ -1708,7 +1711,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13">
       <c r="A2" s="3" t="s">
         <v>3</v>
       </c>
@@ -1745,7 +1748,7 @@
       </c>
       <c r="M2" s="4"/>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13">
       <c r="A3" s="3" t="s">
         <v>5</v>
       </c>
@@ -1780,7 +1783,7 @@
       </c>
       <c r="M3" s="4"/>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13">
       <c r="A4" s="1">
         <v>0</v>
       </c>
@@ -1816,7 +1819,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13">
       <c r="A5" s="1">
         <v>1</v>
       </c>
@@ -1852,7 +1855,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13">
       <c r="A6" s="1">
         <v>2</v>
       </c>
@@ -1888,7 +1891,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13">
       <c r="A7" s="1">
         <v>3</v>
       </c>
@@ -1924,7 +1927,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13">
       <c r="A8" s="1">
         <v>4</v>
       </c>
@@ -1963,7 +1966,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13">
       <c r="A9" s="1">
         <v>5</v>
       </c>
@@ -1999,7 +2002,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13">
       <c r="A10" s="1">
         <v>6</v>
       </c>
@@ -2035,7 +2038,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13">
       <c r="A11" s="1">
         <v>7</v>
       </c>
@@ -2071,7 +2074,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13">
       <c r="A12" s="1">
         <v>8</v>
       </c>
@@ -2110,7 +2113,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13">
       <c r="A13" s="1">
         <v>9</v>
       </c>
@@ -2146,7 +2149,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13">
       <c r="A14" s="1">
         <v>10</v>
       </c>
@@ -2182,7 +2185,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13">
       <c r="A15" s="1">
         <v>11</v>
       </c>
@@ -2218,7 +2221,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13">
       <c r="A16" s="1">
         <v>12</v>
       </c>
@@ -2254,7 +2257,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13">
       <c r="A17" s="1">
         <v>13</v>
       </c>
@@ -2290,7 +2293,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13">
       <c r="A18" s="1">
         <v>14</v>
       </c>
@@ -2326,7 +2329,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13">
       <c r="A19" s="1">
         <v>15</v>
       </c>
@@ -2362,7 +2365,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13">
       <c r="A20" s="1">
         <v>16</v>
       </c>
@@ -2398,7 +2401,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13">
       <c r="A21" s="1">
         <v>17</v>
       </c>
@@ -2434,7 +2437,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13">
       <c r="A22" s="1">
         <v>18</v>
       </c>
@@ -2473,7 +2476,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13">
       <c r="A23" s="1">
         <v>19</v>
       </c>
@@ -2509,7 +2512,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13">
       <c r="A24" s="1">
         <v>20</v>
       </c>
@@ -2545,7 +2548,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13">
       <c r="A25" s="1">
         <v>21</v>
       </c>
@@ -2581,7 +2584,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13">
       <c r="A26" s="1">
         <v>22</v>
       </c>
@@ -2617,7 +2620,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13">
       <c r="A27" s="1">
         <v>23</v>
       </c>
@@ -2653,7 +2656,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:13">
       <c r="A28" s="1">
         <v>24</v>
       </c>
@@ -2692,7 +2695,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:13">
       <c r="A29" s="1">
         <v>25</v>
       </c>
@@ -2731,7 +2734,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:13">
       <c r="A30" s="1">
         <v>26</v>
       </c>
@@ -2767,7 +2770,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:13">
       <c r="A31" s="1">
         <v>27</v>
       </c>
@@ -2803,7 +2806,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:13">
       <c r="A32" s="1">
         <v>28</v>
       </c>
@@ -2842,7 +2845,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:13">
       <c r="A33" s="1">
         <v>29</v>
       </c>
@@ -2890,27 +2893,27 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6FB7AC3-57B9-4D1E-ACF8-A6E6FAE3CA11}">
   <dimension ref="A1:N59"/>
-  <sheetFormatPr defaultRowHeight="12.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="7.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.21875" style="1" customWidth="1"/>
-    <col min="5" max="5" width="16.5546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.44140625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="7.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.25" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.25" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.25" style="1" customWidth="1"/>
+    <col min="5" max="5" width="16.5" style="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.75" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.5" style="1" customWidth="1"/>
     <col min="11" max="11" width="15" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.625" style="1" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="15" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16384" width="8.88671875" style="1"/>
+    <col min="14" max="14" width="9.25" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.25" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16384" width="8.875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14">
       <c r="A1" s="3" t="s">
         <v>2</v>
       </c>
@@ -2954,7 +2957,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14">
       <c r="A2" s="3" t="s">
         <v>3</v>
       </c>
@@ -2996,7 +2999,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14">
       <c r="A3" s="3" t="s">
         <v>5</v>
       </c>
@@ -3036,7 +3039,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14">
       <c r="A4" s="1">
         <v>0</v>
       </c>
@@ -3045,7 +3048,7 @@
       </c>
       <c r="D4" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B4,[2]Material!$B:$B,0))</f>
-        <v>01</v>
+        <v>2F353B</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>190</v>
@@ -3055,7 +3058,7 @@
       </c>
       <c r="G4" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B4,[2]Material!$B:$B,0))</f>
-        <v>230101</v>
+        <v>101001</v>
       </c>
       <c r="H4" s="1">
         <v>10</v>
@@ -3073,7 +3076,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14">
       <c r="A5" s="1">
         <v>1</v>
       </c>
@@ -3082,7 +3085,7 @@
       </c>
       <c r="D5" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B5,[2]Material!$B:$B,0))</f>
-        <v>01</v>
+        <v>E5E4E2</v>
       </c>
       <c r="E5" s="6" t="s">
         <v>190</v>
@@ -3092,7 +3095,7 @@
       </c>
       <c r="G5" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B5,[2]Material!$B:$B,0))</f>
-        <v>230102</v>
+        <v>101002</v>
       </c>
       <c r="H5" s="1">
         <v>10</v>
@@ -3110,7 +3113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14">
       <c r="A6" s="1">
         <v>2</v>
       </c>
@@ -3119,7 +3122,7 @@
       </c>
       <c r="D6" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B6,[2]Material!$B:$B,0))</f>
-        <v>01</v>
+        <v>E34234</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>191</v>
@@ -3129,7 +3132,7 @@
       </c>
       <c r="G6" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B6,[2]Material!$B:$B,0))</f>
-        <v>230103</v>
+        <v>101003</v>
       </c>
       <c r="H6" s="1">
         <v>10</v>
@@ -3147,7 +3150,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14">
       <c r="A7" s="1">
         <v>3</v>
       </c>
@@ -3156,7 +3159,7 @@
       </c>
       <c r="D7" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B7,[2]Material!$B:$B,0))</f>
-        <v>01</v>
+        <v>40E0D0</v>
       </c>
       <c r="E7" s="6" t="s">
         <v>191</v>
@@ -3166,7 +3169,7 @@
       </c>
       <c r="G7" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B7,[2]Material!$B:$B,0))</f>
-        <v>230104</v>
+        <v>101004</v>
       </c>
       <c r="H7" s="1">
         <v>10</v>
@@ -3184,7 +3187,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14">
       <c r="A8" s="1">
         <v>4</v>
       </c>
@@ -3193,7 +3196,7 @@
       </c>
       <c r="D8" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B8,[2]Material!$B:$B,0))</f>
-        <v>01</v>
+        <v>FFFFFF</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>191</v>
@@ -3203,7 +3206,7 @@
       </c>
       <c r="G8" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B8,[2]Material!$B:$B,0))</f>
-        <v>230105</v>
+        <v>101005</v>
       </c>
       <c r="H8" s="1">
         <v>10</v>
@@ -3221,7 +3224,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="13.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:14" ht="15" thickBot="1">
       <c r="A9" s="2">
         <v>5</v>
       </c>
@@ -3230,7 +3233,7 @@
       </c>
       <c r="D9" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B9,[2]Material!$B:$B,0))</f>
-        <v>01</v>
+        <v>FFA500</v>
       </c>
       <c r="E9" s="6" t="s">
         <v>191</v>
@@ -3240,7 +3243,7 @@
       </c>
       <c r="G9" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B9,[2]Material!$B:$B,0))</f>
-        <v>230106</v>
+        <v>101006</v>
       </c>
       <c r="H9" s="1">
         <v>10</v>
@@ -3258,7 +3261,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14">
       <c r="A10" s="1">
         <v>6</v>
       </c>
@@ -3267,7 +3270,7 @@
       </c>
       <c r="D10" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B10,[2]Material!$B:$B,0))</f>
-        <v>01</v>
+        <v>E34234</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>192</v>
@@ -3277,7 +3280,7 @@
       </c>
       <c r="G10" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B10,[2]Material!$B:$B,0))</f>
-        <v>230103</v>
+        <v>101003</v>
       </c>
       <c r="H10" s="1">
         <v>10</v>
@@ -3295,7 +3298,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14">
       <c r="A11" s="1">
         <v>7</v>
       </c>
@@ -3304,7 +3307,7 @@
       </c>
       <c r="D11" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B11,[2]Material!$B:$B,0))</f>
-        <v>01</v>
+        <v>40E0D0</v>
       </c>
       <c r="E11" s="6" t="s">
         <v>192</v>
@@ -3314,7 +3317,7 @@
       </c>
       <c r="G11" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B11,[2]Material!$B:$B,0))</f>
-        <v>230104</v>
+        <v>101004</v>
       </c>
       <c r="H11" s="1">
         <v>10</v>
@@ -3332,7 +3335,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14">
       <c r="A12" s="1">
         <v>8</v>
       </c>
@@ -3341,7 +3344,7 @@
       </c>
       <c r="D12" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B12,[2]Material!$B:$B,0))</f>
-        <v>01</v>
+        <v>FFA500</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>192</v>
@@ -3351,7 +3354,7 @@
       </c>
       <c r="G12" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B12,[2]Material!$B:$B,0))</f>
-        <v>230106</v>
+        <v>101006</v>
       </c>
       <c r="H12" s="1">
         <v>10</v>
@@ -3369,7 +3372,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14">
       <c r="A13" s="1">
         <v>9</v>
       </c>
@@ -3378,7 +3381,7 @@
       </c>
       <c r="D13" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B13,[2]Material!$B:$B,0))</f>
-        <v>02</v>
+        <v>EDEFF2</v>
       </c>
       <c r="E13" s="6" t="s">
         <v>193</v>
@@ -3388,7 +3391,7 @@
       </c>
       <c r="G13" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B13,[2]Material!$B:$B,0))</f>
-        <v>230201</v>
+        <v>102001</v>
       </c>
       <c r="H13" s="1">
         <v>10</v>
@@ -3406,7 +3409,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14">
       <c r="A14" s="1">
         <v>10</v>
       </c>
@@ -3415,7 +3418,7 @@
       </c>
       <c r="D14" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B14,[2]Material!$B:$B,0))</f>
-        <v>02</v>
+        <v>FDFD96</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>193</v>
@@ -3425,7 +3428,7 @@
       </c>
       <c r="G14" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B14,[2]Material!$B:$B,0))</f>
-        <v>230202</v>
+        <v>102002</v>
       </c>
       <c r="H14" s="1">
         <v>10</v>
@@ -3443,7 +3446,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14">
       <c r="A15" s="1">
         <v>11</v>
       </c>
@@ -3455,7 +3458,7 @@
       </c>
       <c r="D15" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B15,[2]Material!$B:$B,0))</f>
-        <v>02</v>
+        <v>FBFBE8</v>
       </c>
       <c r="E15" s="6" t="s">
         <v>193</v>
@@ -3465,7 +3468,7 @@
       </c>
       <c r="G15" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B15,[2]Material!$B:$B,0))</f>
-        <v>230203</v>
+        <v>102003</v>
       </c>
       <c r="H15" s="1">
         <v>10</v>
@@ -3486,7 +3489,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14">
       <c r="A16" s="1">
         <v>12</v>
       </c>
@@ -3495,7 +3498,7 @@
       </c>
       <c r="D16" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B16,[2]Material!$B:$B,0))</f>
-        <v>03</v>
+        <v>FFD700</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>193</v>
@@ -3505,7 +3508,7 @@
       </c>
       <c r="G16" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B16,[2]Material!$B:$B,0))</f>
-        <v>230302</v>
+        <v>103002</v>
       </c>
       <c r="H16" s="1">
         <v>10</v>
@@ -3523,7 +3526,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:14">
       <c r="A17" s="1">
         <v>13</v>
       </c>
@@ -3532,7 +3535,7 @@
       </c>
       <c r="D17" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B17,[2]Material!$B:$B,0))</f>
-        <v>01</v>
+        <v>2F353B</v>
       </c>
       <c r="E17" s="6" t="s">
         <v>194</v>
@@ -3542,7 +3545,7 @@
       </c>
       <c r="G17" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B17,[2]Material!$B:$B,0))</f>
-        <v>230101</v>
+        <v>101001</v>
       </c>
       <c r="H17" s="1">
         <v>10</v>
@@ -3560,7 +3563,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:14">
       <c r="A18" s="1">
         <v>14</v>
       </c>
@@ -3569,7 +3572,7 @@
       </c>
       <c r="D18" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B18,[2]Material!$B:$B,0))</f>
-        <v>01</v>
+        <v>E5E4E2</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>194</v>
@@ -3579,7 +3582,7 @@
       </c>
       <c r="G18" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B18,[2]Material!$B:$B,0))</f>
-        <v>230102</v>
+        <v>101002</v>
       </c>
       <c r="H18" s="1">
         <v>10</v>
@@ -3597,7 +3600,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:14">
       <c r="A19" s="1">
         <v>15</v>
       </c>
@@ -3606,7 +3609,7 @@
       </c>
       <c r="D19" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B19,[2]Material!$B:$B,0))</f>
-        <v>01</v>
+        <v>FFFFFF</v>
       </c>
       <c r="E19" s="6" t="s">
         <v>195</v>
@@ -3616,7 +3619,7 @@
       </c>
       <c r="G19" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B19,[2]Material!$B:$B,0))</f>
-        <v>230105</v>
+        <v>101005</v>
       </c>
       <c r="H19" s="1">
         <v>10</v>
@@ -3634,7 +3637,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:14">
       <c r="A20" s="1">
         <v>16</v>
       </c>
@@ -3646,7 +3649,7 @@
       </c>
       <c r="D20" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B20,[2]Material!$B:$B,0))</f>
-        <v>02</v>
+        <v>FBFBE8</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>195</v>
@@ -3656,7 +3659,7 @@
       </c>
       <c r="G20" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B20,[2]Material!$B:$B,0))</f>
-        <v>230203</v>
+        <v>102003</v>
       </c>
       <c r="H20" s="1">
         <v>10</v>
@@ -3677,7 +3680,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:14" ht="13.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:14" ht="15" thickBot="1">
       <c r="A21" s="2">
         <v>17</v>
       </c>
@@ -3686,7 +3689,7 @@
       </c>
       <c r="D21" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B21,[2]Material!$B:$B,0))</f>
-        <v>03</v>
+        <v>B87333</v>
       </c>
       <c r="E21" s="6" t="s">
         <v>195</v>
@@ -3696,7 +3699,7 @@
       </c>
       <c r="G21" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B21,[2]Material!$B:$B,0))</f>
-        <v>230301</v>
+        <v>103001</v>
       </c>
       <c r="H21" s="1">
         <v>10</v>
@@ -3714,7 +3717,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:14">
       <c r="A22" s="1">
         <v>18</v>
       </c>
@@ -3723,7 +3726,7 @@
       </c>
       <c r="D22" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B22,[2]Material!$B:$B,0))</f>
-        <v>01</v>
+        <v>E34234</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>196</v>
@@ -3733,7 +3736,7 @@
       </c>
       <c r="G22" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B22,[2]Material!$B:$B,0))</f>
-        <v>230103</v>
+        <v>101003</v>
       </c>
       <c r="H22" s="1">
         <v>10</v>
@@ -3751,7 +3754,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:14">
       <c r="A23" s="1">
         <v>19</v>
       </c>
@@ -3760,7 +3763,7 @@
       </c>
       <c r="D23" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B23,[2]Material!$B:$B,0))</f>
-        <v>01</v>
+        <v>FFA500</v>
       </c>
       <c r="E23" s="6" t="s">
         <v>196</v>
@@ -3770,7 +3773,7 @@
       </c>
       <c r="G23" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B23,[2]Material!$B:$B,0))</f>
-        <v>230106</v>
+        <v>101006</v>
       </c>
       <c r="H23" s="1">
         <v>10</v>
@@ -3788,7 +3791,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:14">
       <c r="A24" s="1">
         <v>20</v>
       </c>
@@ -3797,7 +3800,7 @@
       </c>
       <c r="D24" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B24,[2]Material!$B:$B,0))</f>
-        <v>02</v>
+        <v>FDFD96</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>196</v>
@@ -3807,7 +3810,7 @@
       </c>
       <c r="G24" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B24,[2]Material!$B:$B,0))</f>
-        <v>230202</v>
+        <v>102002</v>
       </c>
       <c r="H24" s="1">
         <v>10</v>
@@ -3825,7 +3828,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:14">
       <c r="A25" s="1">
         <v>21</v>
       </c>
@@ -3834,7 +3837,7 @@
       </c>
       <c r="D25" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B25,[2]Material!$B:$B,0))</f>
-        <v>02</v>
+        <v>FBFBE8</v>
       </c>
       <c r="E25" s="6" t="s">
         <v>196</v>
@@ -3844,7 +3847,7 @@
       </c>
       <c r="G25" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B25,[2]Material!$B:$B,0))</f>
-        <v>230203</v>
+        <v>102003</v>
       </c>
       <c r="H25" s="1">
         <v>10</v>
@@ -3862,7 +3865,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:14">
       <c r="A26" s="1">
         <v>22</v>
       </c>
@@ -3871,7 +3874,7 @@
       </c>
       <c r="D26" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B26,[2]Material!$B:$B,0))</f>
-        <v>01</v>
+        <v>40E0D0</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>197</v>
@@ -3881,7 +3884,7 @@
       </c>
       <c r="G26" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B26,[2]Material!$B:$B,0))</f>
-        <v>230104</v>
+        <v>101004</v>
       </c>
       <c r="H26" s="1">
         <v>10</v>
@@ -3899,7 +3902,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:14">
       <c r="A27" s="1">
         <v>23</v>
       </c>
@@ -3908,7 +3911,7 @@
       </c>
       <c r="D27" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B27,[2]Material!$B:$B,0))</f>
-        <v>02</v>
+        <v>EDEFF2</v>
       </c>
       <c r="E27" s="6" t="s">
         <v>197</v>
@@ -3918,7 +3921,7 @@
       </c>
       <c r="G27" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B27,[2]Material!$B:$B,0))</f>
-        <v>230201</v>
+        <v>102001</v>
       </c>
       <c r="H27" s="1">
         <v>10</v>
@@ -3936,7 +3939,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:14">
       <c r="A28" s="1">
         <v>24</v>
       </c>
@@ -3945,7 +3948,7 @@
       </c>
       <c r="D28" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B28,[2]Material!$B:$B,0))</f>
-        <v>01</v>
+        <v>FFFFFF</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>197</v>
@@ -3955,7 +3958,7 @@
       </c>
       <c r="G28" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B28,[2]Material!$B:$B,0))</f>
-        <v>230105</v>
+        <v>101005</v>
       </c>
       <c r="H28" s="1">
         <v>10</v>
@@ -3973,7 +3976,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:14">
       <c r="A29" s="1">
         <v>25</v>
       </c>
@@ -3982,7 +3985,7 @@
       </c>
       <c r="D29" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B29,[2]Material!$B:$B,0))</f>
-        <v>04</v>
+        <v>F5F5F0</v>
       </c>
       <c r="E29" s="6" t="s">
         <v>197</v>
@@ -3992,7 +3995,7 @@
       </c>
       <c r="G29" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B29,[2]Material!$B:$B,0))</f>
-        <v>230401</v>
+        <v>104001</v>
       </c>
       <c r="H29" s="1">
         <v>10</v>
@@ -4010,7 +4013,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:14">
       <c r="A30" s="1">
         <v>26</v>
       </c>
@@ -4019,7 +4022,7 @@
       </c>
       <c r="D30" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B30,[2]Material!$B:$B,0))</f>
-        <v>04</v>
+        <v>E6E8EC</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>197</v>
@@ -4029,7 +4032,7 @@
       </c>
       <c r="G30" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B30,[2]Material!$B:$B,0))</f>
-        <v>230402</v>
+        <v>104002</v>
       </c>
       <c r="H30" s="1">
         <v>10</v>
@@ -4047,7 +4050,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:14">
       <c r="A31" s="1">
         <v>27</v>
       </c>
@@ -4056,7 +4059,7 @@
       </c>
       <c r="D31" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B31,[2]Material!$B:$B,0))</f>
-        <v>04</v>
+        <v>F0F8FF</v>
       </c>
       <c r="E31" s="6" t="s">
         <v>197</v>
@@ -4066,7 +4069,7 @@
       </c>
       <c r="G31" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B31,[2]Material!$B:$B,0))</f>
-        <v>230403</v>
+        <v>104003</v>
       </c>
       <c r="H31" s="1">
         <v>10</v>
@@ -4084,7 +4087,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:14">
       <c r="A32" s="1">
         <v>28</v>
       </c>
@@ -4093,7 +4096,7 @@
       </c>
       <c r="D32" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B32,[2]Material!$B:$B,0))</f>
-        <v>03</v>
+        <v>B87333</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>198</v>
@@ -4103,7 +4106,7 @@
       </c>
       <c r="G32" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B32,[2]Material!$B:$B,0))</f>
-        <v>230301</v>
+        <v>103001</v>
       </c>
       <c r="H32" s="1">
         <v>10</v>
@@ -4121,7 +4124,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:14">
       <c r="A33" s="1">
         <v>29</v>
       </c>
@@ -4130,7 +4133,7 @@
       </c>
       <c r="D33" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B33,[2]Material!$B:$B,0))</f>
-        <v>01</v>
+        <v>2F353B</v>
       </c>
       <c r="E33" s="6" t="s">
         <v>198</v>
@@ -4140,7 +4143,7 @@
       </c>
       <c r="G33" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B33,[2]Material!$B:$B,0))</f>
-        <v>230101</v>
+        <v>101001</v>
       </c>
       <c r="H33" s="1">
         <v>10</v>
@@ -4158,7 +4161,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:14">
       <c r="A34" s="1">
         <v>30</v>
       </c>
@@ -4167,7 +4170,7 @@
       </c>
       <c r="D34" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B34,[2]Material!$B:$B,0))</f>
-        <v>01</v>
+        <v>E5E4E2</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>198</v>
@@ -4177,7 +4180,7 @@
       </c>
       <c r="G34" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B34,[2]Material!$B:$B,0))</f>
-        <v>230102</v>
+        <v>101002</v>
       </c>
       <c r="H34" s="1">
         <v>10</v>
@@ -4195,7 +4198,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:14">
       <c r="A35" s="1">
         <v>31</v>
       </c>
@@ -4204,7 +4207,7 @@
       </c>
       <c r="D35" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B35,[2]Material!$B:$B,0))</f>
-        <v>05</v>
+        <v>4A4A4A</v>
       </c>
       <c r="E35" s="6" t="s">
         <v>199</v>
@@ -4214,7 +4217,7 @@
       </c>
       <c r="G35" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B35,[2]Material!$B:$B,0))</f>
-        <v>230501</v>
+        <v>105001</v>
       </c>
       <c r="H35" s="1">
         <v>10</v>
@@ -4232,7 +4235,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:14">
       <c r="A36" s="1">
         <v>32</v>
       </c>
@@ -4241,7 +4244,7 @@
       </c>
       <c r="D36" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B36,[2]Material!$B:$B,0))</f>
-        <v>05</v>
+        <v>1C1C1C</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>199</v>
@@ -4251,7 +4254,7 @@
       </c>
       <c r="G36" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B36,[2]Material!$B:$B,0))</f>
-        <v>230502</v>
+        <v>105002</v>
       </c>
       <c r="H36" s="1">
         <v>10</v>
@@ -4269,7 +4272,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:14">
       <c r="A37" s="1">
         <v>33</v>
       </c>
@@ -4278,7 +4281,7 @@
       </c>
       <c r="D37" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B37,[2]Material!$B:$B,0))</f>
-        <v>05</v>
+        <v>2FA4A9</v>
       </c>
       <c r="E37" s="6" t="s">
         <v>199</v>
@@ -4288,7 +4291,7 @@
       </c>
       <c r="G37" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B37,[2]Material!$B:$B,0))</f>
-        <v>230504</v>
+        <v>105004</v>
       </c>
       <c r="H37" s="1">
         <v>10</v>
@@ -4306,7 +4309,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:14">
       <c r="A38" s="1">
         <v>34</v>
       </c>
@@ -4315,7 +4318,7 @@
       </c>
       <c r="D38" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B38,[2]Material!$B:$B,0))</f>
-        <v>03</v>
+        <v>FFD700</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>199</v>
@@ -4325,7 +4328,7 @@
       </c>
       <c r="G38" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B38,[2]Material!$B:$B,0))</f>
-        <v>230302</v>
+        <v>103002</v>
       </c>
       <c r="H38" s="1">
         <v>10</v>
@@ -4343,7 +4346,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:14" ht="13.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:14" ht="15" thickBot="1">
       <c r="A39" s="2">
         <v>35</v>
       </c>
@@ -4352,7 +4355,7 @@
       </c>
       <c r="D39" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B39,[2]Material!$B:$B,0))</f>
-        <v>05</v>
+        <v>2B2B2B</v>
       </c>
       <c r="E39" s="6" t="s">
         <v>200</v>
@@ -4362,7 +4365,7 @@
       </c>
       <c r="G39" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B39,[2]Material!$B:$B,0))</f>
-        <v>230503</v>
+        <v>105003</v>
       </c>
       <c r="H39" s="1">
         <v>10</v>
@@ -4380,7 +4383,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:14">
       <c r="A40" s="1">
         <v>36</v>
       </c>
@@ -4389,7 +4392,7 @@
       </c>
       <c r="D40" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B40,[2]Material!$B:$B,0))</f>
-        <v>01</v>
+        <v>E34234</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>201</v>
@@ -4399,7 +4402,7 @@
       </c>
       <c r="G40" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B40,[2]Material!$B:$B,0))</f>
-        <v>230103</v>
+        <v>101003</v>
       </c>
       <c r="H40" s="1">
         <v>10</v>
@@ -4417,7 +4420,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:14">
       <c r="A41" s="1">
         <v>37</v>
       </c>
@@ -4426,7 +4429,7 @@
       </c>
       <c r="D41" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B41,[2]Material!$B:$B,0))</f>
-        <v>01</v>
+        <v>40E0D0</v>
       </c>
       <c r="E41" s="6" t="s">
         <v>201</v>
@@ -4436,7 +4439,7 @@
       </c>
       <c r="G41" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B41,[2]Material!$B:$B,0))</f>
-        <v>230104</v>
+        <v>101004</v>
       </c>
       <c r="H41" s="1">
         <v>10</v>
@@ -4454,7 +4457,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:14">
       <c r="A42" s="1">
         <v>38</v>
       </c>
@@ -4463,7 +4466,7 @@
       </c>
       <c r="D42" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B42,[2]Material!$B:$B,0))</f>
-        <v>02</v>
+        <v>FBFBE8</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>201</v>
@@ -4473,7 +4476,7 @@
       </c>
       <c r="G42" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B42,[2]Material!$B:$B,0))</f>
-        <v>230203</v>
+        <v>102003</v>
       </c>
       <c r="H42" s="1">
         <v>10</v>
@@ -4491,7 +4494,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:14">
       <c r="A43" s="1">
         <v>39</v>
       </c>
@@ -4500,7 +4503,7 @@
       </c>
       <c r="D43" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B43,[2]Material!$B:$B,0))</f>
-        <v>04</v>
+        <v>E6E8EC</v>
       </c>
       <c r="E43" s="6" t="s">
         <v>201</v>
@@ -4510,7 +4513,7 @@
       </c>
       <c r="G43" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B43,[2]Material!$B:$B,0))</f>
-        <v>230402</v>
+        <v>104002</v>
       </c>
       <c r="H43" s="1">
         <v>10</v>
@@ -4528,7 +4531,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:14">
       <c r="A44" s="1">
         <v>40</v>
       </c>
@@ -4537,7 +4540,7 @@
       </c>
       <c r="D44" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B44,[2]Material!$B:$B,0))</f>
-        <v>05</v>
+        <v>4A4A4A</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>201</v>
@@ -4547,7 +4550,7 @@
       </c>
       <c r="G44" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B44,[2]Material!$B:$B,0))</f>
-        <v>230501</v>
+        <v>105001</v>
       </c>
       <c r="H44" s="1">
         <v>10</v>
@@ -4565,7 +4568,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:14">
       <c r="A45" s="1">
         <v>41</v>
       </c>
@@ -4574,7 +4577,7 @@
       </c>
       <c r="D45" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B45,[2]Material!$B:$B,0))</f>
-        <v>04</v>
+        <v>F5F5F0</v>
       </c>
       <c r="E45" s="6" t="s">
         <v>201</v>
@@ -4584,7 +4587,7 @@
       </c>
       <c r="G45" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B45,[2]Material!$B:$B,0))</f>
-        <v>230401</v>
+        <v>104001</v>
       </c>
       <c r="H45" s="1">
         <v>10</v>
@@ -4602,7 +4605,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:14">
       <c r="A46" s="1">
         <v>42</v>
       </c>
@@ -4611,7 +4614,7 @@
       </c>
       <c r="D46" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B46,[2]Material!$B:$B,0))</f>
-        <v>03</v>
+        <v>B87333</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>201</v>
@@ -4621,7 +4624,7 @@
       </c>
       <c r="G46" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B46,[2]Material!$B:$B,0))</f>
-        <v>230301</v>
+        <v>103001</v>
       </c>
       <c r="H46" s="1">
         <v>10</v>
@@ -4639,7 +4642,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:14">
       <c r="A47" s="1">
         <v>43</v>
       </c>
@@ -4648,7 +4651,7 @@
       </c>
       <c r="D47" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B47,[2]Material!$B:$B,0))</f>
-        <v>03</v>
+        <v>FFD700</v>
       </c>
       <c r="E47" s="6" t="s">
         <v>202</v>
@@ -4658,7 +4661,7 @@
       </c>
       <c r="G47" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B47,[2]Material!$B:$B,0))</f>
-        <v>230302</v>
+        <v>103002</v>
       </c>
       <c r="H47" s="1">
         <v>10</v>
@@ -4676,7 +4679,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:14">
       <c r="A48" s="1">
         <v>44</v>
       </c>
@@ -4685,7 +4688,7 @@
       </c>
       <c r="D48" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B48,[2]Material!$B:$B,0))</f>
-        <v>05</v>
+        <v>2FA4A9</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>202</v>
@@ -4695,7 +4698,7 @@
       </c>
       <c r="G48" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B48,[2]Material!$B:$B,0))</f>
-        <v>230504</v>
+        <v>105004</v>
       </c>
       <c r="H48" s="1">
         <v>10</v>
@@ -4713,7 +4716,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:14">
       <c r="A49" s="1">
         <v>45</v>
       </c>
@@ -4722,7 +4725,7 @@
       </c>
       <c r="D49" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B49,[2]Material!$B:$B,0))</f>
-        <v>05</v>
+        <v>1C1C1C</v>
       </c>
       <c r="E49" s="6" t="s">
         <v>202</v>
@@ -4732,7 +4735,7 @@
       </c>
       <c r="G49" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B49,[2]Material!$B:$B,0))</f>
-        <v>230502</v>
+        <v>105002</v>
       </c>
       <c r="H49" s="1">
         <v>10</v>
@@ -4750,7 +4753,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:14">
       <c r="A50" s="1">
         <v>46</v>
       </c>
@@ -4759,7 +4762,7 @@
       </c>
       <c r="D50" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B50,[2]Material!$B:$B,0))</f>
-        <v>04</v>
+        <v>F0F8FF</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>202</v>
@@ -4769,7 +4772,7 @@
       </c>
       <c r="G50" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B50,[2]Material!$B:$B,0))</f>
-        <v>230403</v>
+        <v>104003</v>
       </c>
       <c r="H50" s="1">
         <v>10</v>
@@ -4787,16 +4790,16 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:14">
       <c r="A51" s="1">
         <v>47</v>
       </c>
       <c r="B51" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="D51" s="1" t="str">
+      <c r="D51" s="1">
         <f>INDEX([2]Material!$E:$E,MATCH(B51,[2]Material!$B:$B,0))</f>
-        <v>06</v>
+        <v>800080</v>
       </c>
       <c r="E51" s="6" t="s">
         <v>202</v>
@@ -4806,7 +4809,7 @@
       </c>
       <c r="G51" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B51,[2]Material!$B:$B,0))</f>
-        <v>230601</v>
+        <v>106001</v>
       </c>
       <c r="H51" s="1">
         <v>10</v>
@@ -4824,7 +4827,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:14">
       <c r="A52" s="1">
         <v>48</v>
       </c>
@@ -4833,7 +4836,7 @@
       </c>
       <c r="D52" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B52,[2]Material!$B:$B,0))</f>
-        <v>01</v>
+        <v>FFA500</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>203</v>
@@ -4843,7 +4846,7 @@
       </c>
       <c r="G52" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B52,[2]Material!$B:$B,0))</f>
-        <v>230106</v>
+        <v>101006</v>
       </c>
       <c r="H52" s="1">
         <v>10</v>
@@ -4861,7 +4864,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:14">
       <c r="A53" s="1">
         <v>49</v>
       </c>
@@ -4870,7 +4873,7 @@
       </c>
       <c r="D53" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B53,[2]Material!$B:$B,0))</f>
-        <v>02</v>
+        <v>FDFD96</v>
       </c>
       <c r="E53" s="6" t="s">
         <v>203</v>
@@ -4880,7 +4883,7 @@
       </c>
       <c r="G53" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B53,[2]Material!$B:$B,0))</f>
-        <v>230202</v>
+        <v>102002</v>
       </c>
       <c r="H53" s="1">
         <v>10</v>
@@ -4898,7 +4901,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:14">
       <c r="A54" s="1">
         <v>50</v>
       </c>
@@ -4907,7 +4910,7 @@
       </c>
       <c r="D54" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B54,[2]Material!$B:$B,0))</f>
-        <v>02</v>
+        <v>EDEFF2</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>203</v>
@@ -4917,7 +4920,7 @@
       </c>
       <c r="G54" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B54,[2]Material!$B:$B,0))</f>
-        <v>230201</v>
+        <v>102001</v>
       </c>
       <c r="H54" s="1">
         <v>10</v>
@@ -4935,7 +4938,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:14">
       <c r="A55" s="1">
         <v>51</v>
       </c>
@@ -4944,7 +4947,7 @@
       </c>
       <c r="D55" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B55,[2]Material!$B:$B,0))</f>
-        <v>01</v>
+        <v>FFFFFF</v>
       </c>
       <c r="E55" s="6" t="s">
         <v>203</v>
@@ -4954,7 +4957,7 @@
       </c>
       <c r="G55" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B55,[2]Material!$B:$B,0))</f>
-        <v>230105</v>
+        <v>101005</v>
       </c>
       <c r="H55" s="1">
         <v>10</v>
@@ -4972,7 +4975,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:14">
       <c r="A56" s="1">
         <v>52</v>
       </c>
@@ -4981,7 +4984,7 @@
       </c>
       <c r="D56" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B56,[2]Material!$B:$B,0))</f>
-        <v>01</v>
+        <v>2F353B</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>204</v>
@@ -4991,7 +4994,7 @@
       </c>
       <c r="G56" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B56,[2]Material!$B:$B,0))</f>
-        <v>230101</v>
+        <v>101001</v>
       </c>
       <c r="H56" s="1">
         <v>10</v>
@@ -5009,7 +5012,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:14">
       <c r="A57" s="1">
         <v>53</v>
       </c>
@@ -5018,7 +5021,7 @@
       </c>
       <c r="D57" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B57,[2]Material!$B:$B,0))</f>
-        <v>01</v>
+        <v>E5E4E2</v>
       </c>
       <c r="E57" s="6" t="s">
         <v>204</v>
@@ -5028,7 +5031,7 @@
       </c>
       <c r="G57" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B57,[2]Material!$B:$B,0))</f>
-        <v>230102</v>
+        <v>101002</v>
       </c>
       <c r="H57" s="1">
         <v>10</v>
@@ -5046,7 +5049,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:14">
       <c r="A58" s="1">
         <v>54</v>
       </c>
@@ -5055,7 +5058,7 @@
       </c>
       <c r="D58" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B58,[2]Material!$B:$B,0))</f>
-        <v>05</v>
+        <v>2B2B2B</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>204</v>
@@ -5065,7 +5068,7 @@
       </c>
       <c r="G58" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B58,[2]Material!$B:$B,0))</f>
-        <v>230503</v>
+        <v>105003</v>
       </c>
       <c r="H58" s="1">
         <v>10</v>
@@ -5083,7 +5086,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:14" ht="13.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:14" ht="15" thickBot="1">
       <c r="A59" s="2">
         <v>55</v>
       </c>
@@ -5092,7 +5095,7 @@
       </c>
       <c r="D59" s="1" t="str">
         <f>INDEX([2]Material!$E:$E,MATCH(B59,[2]Material!$B:$B,0))</f>
-        <v>06</v>
+        <v>9C3A2B</v>
       </c>
       <c r="E59" s="6" t="s">
         <v>204</v>
@@ -5102,7 +5105,7 @@
       </c>
       <c r="G59" s="1" t="str">
         <f>INDEX([2]Material!$C:$C,MATCH($B59,[2]Material!$B:$B,0))</f>
-        <v>230602</v>
+        <v>106002</v>
       </c>
       <c r="H59" s="1">
         <v>10</v>

</xml_diff>